<commit_message>
Merge unified news results: resume-8ace4fc710054c79af17e3416a397b99
</commit_message>
<xml_diff>
--- a/news_daily/2026-10-24.xlsx
+++ b/news_daily/2026-10-24.xlsx
@@ -16,9 +16,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'完整新聞'!$A$1:$AW$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主要負面事件'!$A$1:$AW$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待人工覆核'!$A$1:$AW$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待補分析'!$A$1:$AW$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'執行紀錄'!$A$1:$W$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待人工覆核'!$A$1:$AW$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待補分析'!$A$1:$AW$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'執行紀錄'!$A$1:$W$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -779,18 +779,22 @@
           <t>格隆匯快訊</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>目前無足夠資訊判斷 Meta Platforms 是否存在信用風險事件。</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>待補分析</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>待補分析</t>
+          <t>待人工覆核</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -803,8 +807,10 @@
           <t>方法一</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>-0.023</v>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>'-0.023</t>
+        </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -813,7 +819,11 @@
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>公司清單／原始紀錄</t>
@@ -841,16 +851,24 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>QUOTA_PENDING</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AI2" s="2" t="inlineStr">
@@ -863,8 +881,12 @@
           <t>financial_events_v1.0</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr"/>
-      <c r="AL2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="n">
+        <v>1436</v>
+      </c>
+      <c r="AL2" s="2" t="n">
+        <v>88</v>
+      </c>
       <c r="AM2" s="2" t="inlineStr"/>
       <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr">
@@ -885,12 +907,12 @@
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr">
         <is>
-          <t>e694e02ebc43cdbf2152a98a6a76d3b86bee99fe2841dd3ba80e548b1afb8f90</t>
+          <t>f80136a94c40ca97648545179781402c508a2190f1e5997765e9ff086f7a0ef5</t>
         </is>
       </c>
       <c r="AT2" s="2" t="inlineStr">
         <is>
-          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
+          <t>resume-8ace4fc710054c79af17e3416a397b99</t>
         </is>
       </c>
       <c r="AU2" s="2" t="inlineStr">
@@ -1230,6 +1252,498 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AW2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="65" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="65" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="37" max="37"/>
+    <col width="22" customWidth="1" min="38" max="38"/>
+    <col width="22" customWidth="1" min="39" max="39"/>
+    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="22" customWidth="1" min="41" max="41"/>
+    <col width="22" customWidth="1" min="42" max="42"/>
+    <col width="22" customWidth="1" min="43" max="43"/>
+    <col width="22" customWidth="1" min="44" max="44"/>
+    <col width="22" customWidth="1" min="45" max="45"/>
+    <col width="22" customWidth="1" min="46" max="46"/>
+    <col width="22" customWidth="1" min="47" max="47"/>
+    <col width="22" customWidth="1" min="48" max="48"/>
+    <col width="22" customWidth="1" min="49" max="49"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Published Time</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>中文摘要</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>事件中文</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>最終判斷來源</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>分類狀態</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>已人工覆核</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>來源方法</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FinBERT</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_Event_Code</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_Level</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>LLM事件代碼</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>LLM辨識公司</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker來源</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>news_id</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>監控池</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword候選</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword事件代碼</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>LLM狀態</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>事件狀態</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed_Default</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Event_Code</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>需要人工覆核</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>LLM模型</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt版本</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>API錯誤</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>人工版本</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_Action</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_事件中文</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Exchange</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>分析指紋</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>最近執行</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Title_ZH</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>FinBERT_Title</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>分析快取</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:04:58+08:00</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>格隆匯快訊</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>目前無足夠資訊判斷 Meta Platforms 是否存在信用風險事件。</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>待人工覆核</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>方法一</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>'-0.023</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>公司清單／原始紀錄</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gelonghui.com/live/2727118</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>TradingView</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>6ed3a0fe8361517af740a8e3</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>financial_events_v1.0</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="n">
+        <v>1436</v>
+      </c>
+      <c r="AL2" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AN2" s="2" t="inlineStr"/>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>ccef7cb36f86f9aa2bbaa569</t>
+        </is>
+      </c>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>人工確認</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>待人工覆核</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr"/>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>f80136a94c40ca97648545179781402c508a2190f1e5997765e9ff086f7a0ef5</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>resume-8ace4fc710054c79af17e3416a397b99</t>
+        </is>
+      </c>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>格隆匯快訊</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>Gelonghui News</t>
+        </is>
+      </c>
+      <c r="AW2" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AW2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1537,483 +2051,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AW2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="65" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="22" customWidth="1" min="29" max="29"/>
-    <col width="22" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="65" customWidth="1" min="32" max="32"/>
-    <col width="22" customWidth="1" min="33" max="33"/>
-    <col width="22" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
-    <col width="22" customWidth="1" min="36" max="36"/>
-    <col width="22" customWidth="1" min="37" max="37"/>
-    <col width="22" customWidth="1" min="38" max="38"/>
-    <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
-    <col width="22" customWidth="1" min="41" max="41"/>
-    <col width="22" customWidth="1" min="42" max="42"/>
-    <col width="22" customWidth="1" min="43" max="43"/>
-    <col width="22" customWidth="1" min="44" max="44"/>
-    <col width="22" customWidth="1" min="45" max="45"/>
-    <col width="22" customWidth="1" min="46" max="46"/>
-    <col width="22" customWidth="1" min="47" max="47"/>
-    <col width="22" customWidth="1" min="48" max="48"/>
-    <col width="22" customWidth="1" min="49" max="49"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Market</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Published Time</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>中文摘要</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>事件中文</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>最終判斷來源</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>分類狀態</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>已人工覆核</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>來源方法</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>FinBERT</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_Event_Code</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_Level</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>LLM事件代碼</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>LLM辨識公司</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker來源</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>news_id</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Language</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>監控池</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Keyword候選</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Keyword事件代碼</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>LLM狀態</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>事件狀態</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Confirmed_Default</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Event_Code</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>需要人工覆核</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>LLM模型</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>Prompt版本</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>input_tokens</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>output_tokens</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>API錯誤</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>人工版本</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>article_id</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_Action</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_事件中文</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>Exchange</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>分析指紋</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>最近執行</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Title_ZH</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>FinBERT_Title</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>分析快取</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Meta Platforms</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:04:58+08:00</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>格隆匯快訊</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>待補分析</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>待補分析</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>方法一</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>-0.023</v>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>公司清單／原始紀錄</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gelonghui.com/live/2727118</t>
-        </is>
-      </c>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>TradingView</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>6ed3a0fe8361517af740a8e3</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr"/>
-      <c r="Y2" s="2" t="inlineStr"/>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="inlineStr"/>
-      <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr">
-        <is>
-          <t>QUOTA_PENDING</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr"/>
-      <c r="AF2" s="2" t="inlineStr"/>
-      <c r="AG2" s="2" t="inlineStr"/>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>openai/gpt-oss-20b</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>financial_events_v1.0</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr"/>
-      <c r="AL2" s="2" t="inlineStr"/>
-      <c r="AM2" s="2" t="inlineStr"/>
-      <c r="AN2" s="2" t="inlineStr"/>
-      <c r="AO2" s="2" t="inlineStr">
-        <is>
-          <t>ccef7cb36f86f9aa2bbaa569</t>
-        </is>
-      </c>
-      <c r="AP2" s="2" t="inlineStr">
-        <is>
-          <t>人工確認</t>
-        </is>
-      </c>
-      <c r="AQ2" s="2" t="inlineStr">
-        <is>
-          <t>待人工覆核</t>
-        </is>
-      </c>
-      <c r="AR2" s="2" t="inlineStr"/>
-      <c r="AS2" s="2" t="inlineStr">
-        <is>
-          <t>e694e02ebc43cdbf2152a98a6a76d3b86bee99fe2841dd3ba80e548b1afb8f90</t>
-        </is>
-      </c>
-      <c r="AT2" s="2" t="inlineStr">
-        <is>
-          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
-        </is>
-      </c>
-      <c r="AU2" s="2" t="inlineStr">
-        <is>
-          <t>格隆匯快訊</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
-        <is>
-          <t>Gelonghui News</t>
-        </is>
-      </c>
-      <c r="AW2" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:AW2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2161,7 +2205,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
+          <t>resume-8ace4fc710054c79af17e3416a397b99</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2176,12 +2220,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T00:16:00+08:00</t>
+          <t>2026-10-22T00:26:32.508450+08:00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:16:00+08:00</t>
+          <t>2026-10-24T00:26:32.508450+08:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -2189,47 +2233,43 @@
           <t>US</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>方法一|方法二</t>
-        </is>
-      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:20:47.845317+08:00</t>
+          <t>2026-10-24T00:26:34.299718+08:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:21:20.302846+08:00</t>
+          <t>2026-10-24T00:32:11.776786+08:00</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="O2" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="P2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
@@ -2238,14 +2278,14 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>['方法一 6 筆', '方法二 12 筆；公司 1 家（非輪替）', 'FinBERT 完成 18 筆']</t>
+          <t>['沿用已擷取資料；不重新抓取']</t>
         </is>
       </c>
       <c r="U2" s="2" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="W2" s="2" t="n">
         <v>0</v>
@@ -2254,7 +2294,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>a62af6ad2a0044b7a685a4178159b27a</t>
+          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2292,37 +2332,37 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:19:11.949238+08:00</t>
+          <t>2026-10-24T00:20:47.845317+08:00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:19:18.833437+08:00</t>
+          <t>2026-10-24T00:21:20.302846+08:00</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
@@ -2331,21 +2371,114 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>['沿用已擷取資料；不重新抓取']</t>
+          <t>['方法一 6 筆', '方法二 12 筆；公司 1 家（非輪替）', 'FinBERT 完成 18 筆']</t>
         </is>
       </c>
       <c r="U3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="W3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>a62af6ad2a0044b7a685a4178159b27a</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T00:16:00+08:00</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:16:00+08:00</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>方法一|方法二</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:19:11.949238+08:00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:19:18.833437+08:00</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>['沿用已擷取資料；不重新抓取']</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W3"/>
+  <autoFilter ref="A1:W4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audit and backfill verified tickers across all stored news dates
</commit_message>
<xml_diff>
--- a/news_daily/2026-10-24.xlsx
+++ b/news_daily/2026-10-24.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="執行紀錄" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'完整新聞'!$A$1:$AW$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主要負面事件'!$A$1:$AW$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待人工覆核'!$A$1:$AW$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待補分析'!$A$1:$AW$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'執行紀錄'!$A$1:$W$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'完整新聞'!$A$1:$BH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主要負面事件'!$A$1:$BH$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待人工覆核'!$A$1:$BH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待補分析'!$A$1:$BH$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'執行紀錄'!$A$1:$AA$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW2"/>
+  <dimension ref="A1:BH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="65" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
@@ -489,7 +489,7 @@
     <col width="22" customWidth="1" min="37" max="37"/>
     <col width="22" customWidth="1" min="38" max="38"/>
     <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="65" customWidth="1" min="40" max="40"/>
     <col width="22" customWidth="1" min="41" max="41"/>
     <col width="22" customWidth="1" min="42" max="42"/>
     <col width="22" customWidth="1" min="43" max="43"/>
@@ -499,6 +499,17 @@
     <col width="22" customWidth="1" min="47" max="47"/>
     <col width="22" customWidth="1" min="48" max="48"/>
     <col width="22" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="22" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="22" customWidth="1" min="54" max="54"/>
+    <col width="22" customWidth="1" min="55" max="55"/>
+    <col width="22" customWidth="1" min="56" max="56"/>
+    <col width="22" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
+    <col width="22" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,137 +625,192 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Title_ZH</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Event_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Event_Code</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>人工版本</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>news_id</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>監控池</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>監控池</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Keyword候選</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Keyword事件代碼</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LLM狀態</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>事件狀態</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Confirmed_Default</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Event_Code</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>需要人工覆核</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>LLM模型</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Prompt版本</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>API錯誤</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>人工版本</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>article_id</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Rule_Action</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Rule_事件中文</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Exchange</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>分析指紋</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>最近執行</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Title_ZH</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>FinBERT_Title</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>分析快取</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>原始Ticker</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker狀態</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker候選</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker核對依據</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker參照日期</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>上市狀態</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker稽核警示</t>
         </is>
       </c>
     </row>
@@ -759,11 +825,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
@@ -826,7 +888,7 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>公司清單／原始紀錄</t>
+          <t>主體證據不足</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
@@ -841,7 +903,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>6ed3a0fe8361517af740a8e3</t>
+          <t>格隆匯快訊</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr"/>
@@ -851,84 +913,119 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ccef7cb36f86f9aa2bbaa569</t>
         </is>
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>UNCLEAR</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
+          <t>6ed3a0fe8361517af740a8e3</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>openai/gpt-oss-20b</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>financial_events_v1.0</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="n">
-        <v>1436</v>
-      </c>
-      <c r="AL2" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr">
         <is>
-          <t>ccef7cb36f86f9aa2bbaa569</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AP2" s="2" t="inlineStr">
         <is>
+          <t>openai/gpt-oss-20b</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>financial_events_v1.0</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>1436</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
           <t>人工確認</t>
         </is>
       </c>
-      <c r="AQ2" s="2" t="inlineStr">
+      <c r="AV2" s="2" t="inlineStr">
         <is>
           <t>待人工覆核</t>
         </is>
       </c>
-      <c r="AR2" s="2" t="inlineStr"/>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="AX2" s="2" t="inlineStr">
         <is>
           <t>f80136a94c40ca97648545179781402c508a2190f1e5997765e9ff086f7a0ef5</t>
         </is>
       </c>
-      <c r="AT2" s="2" t="inlineStr">
+      <c r="AY2" s="2" t="inlineStr">
         <is>
           <t>resume-8ace4fc710054c79af17e3416a397b99</t>
         </is>
       </c>
-      <c r="AU2" s="2" t="inlineStr">
-        <is>
-          <t>格隆匯快訊</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
+      <c r="AZ2" s="2" t="inlineStr">
         <is>
           <t>Gelonghui News</t>
         </is>
       </c>
-      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="BA2" s="2" t="inlineStr"/>
+      <c r="BB2" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="BC2" s="2" t="inlineStr">
+        <is>
+          <t>主體證據不足</t>
+        </is>
+      </c>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>https://investor.atmeta.com/stock-info/default.aspx</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr"/>
+      <c r="BH2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW2"/>
+  <autoFilter ref="A1:BH2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -939,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1"/>
+  <dimension ref="A1:BH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -973,7 +1070,7 @@
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="65" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
@@ -981,7 +1078,7 @@
     <col width="22" customWidth="1" min="37" max="37"/>
     <col width="22" customWidth="1" min="38" max="38"/>
     <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="65" customWidth="1" min="40" max="40"/>
     <col width="22" customWidth="1" min="41" max="41"/>
     <col width="22" customWidth="1" min="42" max="42"/>
     <col width="22" customWidth="1" min="43" max="43"/>
@@ -991,6 +1088,17 @@
     <col width="22" customWidth="1" min="47" max="47"/>
     <col width="22" customWidth="1" min="48" max="48"/>
     <col width="22" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="22" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="22" customWidth="1" min="54" max="54"/>
+    <col width="22" customWidth="1" min="55" max="55"/>
+    <col width="22" customWidth="1" min="56" max="56"/>
+    <col width="22" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
+    <col width="22" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1106,142 +1214,197 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Title_ZH</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Event_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Event_Code</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>人工版本</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>news_id</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>監控池</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>監控池</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Keyword候選</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Keyword事件代碼</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LLM狀態</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>事件狀態</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Confirmed_Default</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Event_Code</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>需要人工覆核</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>LLM模型</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Prompt版本</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>API錯誤</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>人工版本</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>article_id</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Rule_Action</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Rule_事件中文</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Exchange</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>分析指紋</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>最近執行</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Title_ZH</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>FinBERT_Title</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>分析快取</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>原始Ticker</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker狀態</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker候選</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker核對依據</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker參照日期</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>上市狀態</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker稽核警示</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW1"/>
+  <autoFilter ref="A1:BH1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1252,7 +1415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW2"/>
+  <dimension ref="A1:BH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1286,7 +1449,7 @@
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="65" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
@@ -1294,7 +1457,7 @@
     <col width="22" customWidth="1" min="37" max="37"/>
     <col width="22" customWidth="1" min="38" max="38"/>
     <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="65" customWidth="1" min="40" max="40"/>
     <col width="22" customWidth="1" min="41" max="41"/>
     <col width="22" customWidth="1" min="42" max="42"/>
     <col width="22" customWidth="1" min="43" max="43"/>
@@ -1304,6 +1467,17 @@
     <col width="22" customWidth="1" min="47" max="47"/>
     <col width="22" customWidth="1" min="48" max="48"/>
     <col width="22" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="22" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="22" customWidth="1" min="54" max="54"/>
+    <col width="22" customWidth="1" min="55" max="55"/>
+    <col width="22" customWidth="1" min="56" max="56"/>
+    <col width="22" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
+    <col width="22" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1419,137 +1593,192 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Title_ZH</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Event_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Event_Code</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>人工版本</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>news_id</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>監控池</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>監控池</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Keyword候選</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Keyword事件代碼</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LLM狀態</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>事件狀態</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Confirmed_Default</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Event_Code</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>需要人工覆核</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>LLM模型</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Prompt版本</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>API錯誤</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>人工版本</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>article_id</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Rule_Action</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Rule_事件中文</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Exchange</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>分析指紋</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>最近執行</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Title_ZH</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>FinBERT_Title</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>分析快取</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>原始Ticker</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker狀態</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker候選</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker核對依據</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker參照日期</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>上市狀態</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker稽核警示</t>
         </is>
       </c>
     </row>
@@ -1564,11 +1793,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
@@ -1631,7 +1856,7 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>公司清單／原始紀錄</t>
+          <t>主體證據不足</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
@@ -1646,7 +1871,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>6ed3a0fe8361517af740a8e3</t>
+          <t>格隆匯快訊</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr"/>
@@ -1656,84 +1881,119 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ccef7cb36f86f9aa2bbaa569</t>
         </is>
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>UNCLEAR</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
+          <t>6ed3a0fe8361517af740a8e3</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>openai/gpt-oss-20b</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>financial_events_v1.0</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="n">
-        <v>1436</v>
-      </c>
-      <c r="AL2" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr">
         <is>
-          <t>ccef7cb36f86f9aa2bbaa569</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AP2" s="2" t="inlineStr">
         <is>
+          <t>openai/gpt-oss-20b</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>financial_events_v1.0</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>1436</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
           <t>人工確認</t>
         </is>
       </c>
-      <c r="AQ2" s="2" t="inlineStr">
+      <c r="AV2" s="2" t="inlineStr">
         <is>
           <t>待人工覆核</t>
         </is>
       </c>
-      <c r="AR2" s="2" t="inlineStr"/>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="AX2" s="2" t="inlineStr">
         <is>
           <t>f80136a94c40ca97648545179781402c508a2190f1e5997765e9ff086f7a0ef5</t>
         </is>
       </c>
-      <c r="AT2" s="2" t="inlineStr">
+      <c r="AY2" s="2" t="inlineStr">
         <is>
           <t>resume-8ace4fc710054c79af17e3416a397b99</t>
         </is>
       </c>
-      <c r="AU2" s="2" t="inlineStr">
-        <is>
-          <t>格隆匯快訊</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
+      <c r="AZ2" s="2" t="inlineStr">
         <is>
           <t>Gelonghui News</t>
         </is>
       </c>
-      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="BA2" s="2" t="inlineStr"/>
+      <c r="BB2" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="BC2" s="2" t="inlineStr">
+        <is>
+          <t>主體證據不足</t>
+        </is>
+      </c>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>https://investor.atmeta.com/stock-info/default.aspx</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr"/>
+      <c r="BH2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW2"/>
+  <autoFilter ref="A1:BH2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1744,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1"/>
+  <dimension ref="A1:BH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1778,7 +2038,7 @@
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="65" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
@@ -1786,7 +2046,7 @@
     <col width="22" customWidth="1" min="37" max="37"/>
     <col width="22" customWidth="1" min="38" max="38"/>
     <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="65" customWidth="1" min="40" max="40"/>
     <col width="22" customWidth="1" min="41" max="41"/>
     <col width="22" customWidth="1" min="42" max="42"/>
     <col width="22" customWidth="1" min="43" max="43"/>
@@ -1796,6 +2056,17 @@
     <col width="22" customWidth="1" min="47" max="47"/>
     <col width="22" customWidth="1" min="48" max="48"/>
     <col width="22" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="22" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="22" customWidth="1" min="54" max="54"/>
+    <col width="22" customWidth="1" min="55" max="55"/>
+    <col width="22" customWidth="1" min="56" max="56"/>
+    <col width="22" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
+    <col width="22" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1911,142 +2182,197 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Title_ZH</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Event_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Event_Code</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>人工版本</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>news_id</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>監控池</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>監控池</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Keyword候選</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Keyword事件代碼</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LLM狀態</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>事件狀態</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Confirmed_Default</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Event_Code</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>需要人工覆核</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>LLM模型</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Prompt版本</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>API錯誤</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>人工版本</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>article_id</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Rule_Action</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Rule_事件中文</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Exchange</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>分析指紋</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>最近執行</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Title_ZH</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>FinBERT_Title</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>分析快取</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>原始Ticker</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker狀態</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker候選</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker核對依據</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker參照日期</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>上市狀態</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker稽核警示</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW1"/>
+  <autoFilter ref="A1:BH1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2057,7 +2383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2083,6 +2409,10 @@
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2103,100 +2433,120 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>finished_at</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>changed</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>missing_publication_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ticker_statuses</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>llm_calls</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>start</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>market</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>methods</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ai</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>finished_at</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>llm_calls</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>cache_reused</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>review</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>major</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>selected_company_count</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>collected</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>rows</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>errors</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>stages</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>quota_reserved</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>重複合併</t>
         </is>
@@ -2205,12 +2555,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>resume-8ace4fc710054c79af17e3416a397b99</t>
+          <t>ticker-audit-20261024-081549</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ticker-audit</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2220,81 +2570,55 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T00:26:32.508450+08:00</t>
+          <t>2026-10-24T08:15:49.296780+08:00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:26:32.508450+08:00</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:26:34.299718+08:00</t>
-        </is>
+          <t>2026-10-24T08:15:49.296790+08:00</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1691</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>257</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:32:11.776786+08:00</t>
+          <t>{'已核對': 1429, '主體證據不足': 218, '人工確認': 20, '市場／多公司或主體待辨識': 10, '公司名稱／股票代號歧義': 7, '公司代號待核對': 4, '非本市場上市主體': 2, '非上市機構': 1}</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="M2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>['沿用已擷取資料；不重新抓取']</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
+          <t>resume-8ace4fc710054c79af17e3416a397b99</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2309,85 +2633,85 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T00:16:00+08:00</t>
+          <t>2026-10-24T00:26:34.299718+08:00</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:16:00+08:00</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+          <t>2026-10-24T00:32:11.776786+08:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22T00:26:32.508450+08:00</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:26:32.508450+08:00</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>方法一|方法二</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="b">
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:20:47.845317+08:00</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:21:20.302846+08:00</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M3" s="2" t="n">
+      <c r="Q3" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="T3" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="N3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="R3" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>['方法一 6 筆', '方法二 12 筆；公司 1 家（非輪替）', 'FinBERT 完成 18 筆']</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V3" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="W3" s="2" t="n">
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>['沿用已擷取資料；不重新抓取']</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>a62af6ad2a0044b7a685a4178159b27a</t>
+          <t>044ceacec26a4a2f8d3d0f4d45d89e7a</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2402,83 +2726,184 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>2026-10-24T00:20:47.845317+08:00</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:21:20.302846+08:00</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
           <t>2026-10-23T00:16:00+08:00</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>2026-10-24T00:16:00+08:00</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>方法一|方法二</t>
         </is>
       </c>
-      <c r="H4" s="2" t="b">
+      <c r="P4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:19:11.949238+08:00</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T00:19:18.833437+08:00</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="O4" s="2" t="n">
+      <c r="Q4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="P4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>['沿用已擷取資料；不重新抓取']</t>
-        </is>
+      <c r="S4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="U4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V4" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>['方法一 6 筆', '方法二 12 筆；公司 1 家（非輪替）', 'FinBERT 完成 18 筆']</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="W4" s="2" t="n">
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>a62af6ad2a0044b7a685a4178159b27a</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:19:11.949238+08:00</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:19:18.833437+08:00</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T00:16:00+08:00</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T00:16:00+08:00</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>方法一|方法二</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>['沿用已擷取資料；不重新抓取']</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="2" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W4"/>
+  <autoFilter ref="A1:AA5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>